<commit_message>
Aktualizace katalogu produktů - 23.08.2026 14:41
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G553"/>
+  <dimension ref="A1:G556"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14469,6 +14469,81 @@
       </c>
       <c r="G553" t="inlineStr"/>
     </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>Dětská postel se zábranou BASIC GUARD vč. roštu</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>T.ROZOWE 1/3</t>
+        </is>
+      </c>
+      <c r="C554" t="n">
+        <v>21</v>
+      </c>
+      <c r="D554" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E554" t="n">
+        <v>95</v>
+      </c>
+      <c r="F554" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G554" t="inlineStr"/>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>Dětská postel se zábranou BASIC GUARD vč. roštu</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>T.ROZOWE 2/3</t>
+        </is>
+      </c>
+      <c r="C555" t="n">
+        <v>30</v>
+      </c>
+      <c r="D555" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E555" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F555" t="n">
+        <v>1</v>
+      </c>
+      <c r="G555" t="inlineStr"/>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>Dětská postel se zábranou BASIC GUARD vč. roštu</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>T.ROZOWE 3/3</t>
+        </is>
+      </c>
+      <c r="C556" t="n">
+        <v>2</v>
+      </c>
+      <c r="D556" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E556" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F556" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G556" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 23.08.2026 14:42
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G558"/>
+  <dimension ref="A1:G559"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14594,6 +14594,31 @@
       </c>
       <c r="G558" t="inlineStr"/>
     </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>Sendvičová matrace OLIVER výška 11 cm</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>PALIEND</t>
+        </is>
+      </c>
+      <c r="C559" t="n">
+        <v>10</v>
+      </c>
+      <c r="D559" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="E559" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F559" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G559" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 23.08.2026 14:43
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G560"/>
+  <dimension ref="A1:G563"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14644,6 +14644,81 @@
       </c>
       <c r="G560" t="inlineStr"/>
     </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 200x200 masiv borovice - VMK2A</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>VMK2A-200 1/3</t>
+        </is>
+      </c>
+      <c r="C561" t="n">
+        <v>8</v>
+      </c>
+      <c r="D561" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="E561" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F561" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="G561" t="inlineStr"/>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 200x200 masiv borovice - VMK2A</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>VMK2A-200 2/3</t>
+        </is>
+      </c>
+      <c r="C562" t="n">
+        <v>12</v>
+      </c>
+      <c r="D562" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E562" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F562" t="n">
+        <v>2</v>
+      </c>
+      <c r="G562" t="inlineStr"/>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 200x200 masiv borovice - VMK2A</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>VMK2A-200 3/3</t>
+        </is>
+      </c>
+      <c r="C563" t="n">
+        <v>10</v>
+      </c>
+      <c r="D563" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E563" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="F563" t="n">
+        <v>1</v>
+      </c>
+      <c r="G563" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 23.08.2026 14:55
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G563"/>
+  <dimension ref="A1:G566"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14719,6 +14719,81 @@
       </c>
       <c r="G563" t="inlineStr"/>
     </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>Patrová postel PP06, se zábranou  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>LP06 1/3</t>
+        </is>
+      </c>
+      <c r="C564" t="n">
+        <v>19</v>
+      </c>
+      <c r="D564" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E564" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F564" t="n">
+        <v>1</v>
+      </c>
+      <c r="G564" t="inlineStr"/>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>Patrová postel PP06, se zábranou  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>LP06 2/3</t>
+        </is>
+      </c>
+      <c r="C565" t="n">
+        <v>27</v>
+      </c>
+      <c r="D565" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E565" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F565" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G565" t="inlineStr"/>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>Patrová postel PP06, se zábranou  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>LP06 3/3</t>
+        </is>
+      </c>
+      <c r="C566" t="n">
+        <v>24</v>
+      </c>
+      <c r="D566" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E566" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F566" t="n">
+        <v>1</v>
+      </c>
+      <c r="G566" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 23.08.2026 14:58
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G566"/>
+  <dimension ref="A1:G568"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14794,6 +14794,56 @@
       </c>
       <c r="G566" t="inlineStr"/>
     </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>Patrová postel ZP04, vyvýšené patro</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>ZP04 1/2</t>
+        </is>
+      </c>
+      <c r="C567" t="n">
+        <v>24</v>
+      </c>
+      <c r="D567" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E567" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F567" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G567" t="inlineStr"/>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>Patrová postel ZP04, vyvýšené patro</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>ZP04 2/2</t>
+        </is>
+      </c>
+      <c r="C568" t="n">
+        <v>22</v>
+      </c>
+      <c r="D568" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E568" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F568" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G568" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 24.08.2026 10:23
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G568"/>
+  <dimension ref="A1:G572"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14844,6 +14844,106 @@
       </c>
       <c r="G568" t="inlineStr"/>
     </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>Obývací stěna TERA | ŠEDÝ BETON / BÍLÁ</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>STĚNA-TERA 1/4</t>
+        </is>
+      </c>
+      <c r="C569" t="n">
+        <v>18</v>
+      </c>
+      <c r="D569" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E569" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F569" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="G569" t="inlineStr"/>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>Obývací stěna TERA | ŠEDÝ BETON / BÍLÁ</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>STĚNA-TERA 2/4</t>
+        </is>
+      </c>
+      <c r="C570" t="n">
+        <v>8</v>
+      </c>
+      <c r="D570" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E570" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="F570" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G570" t="inlineStr"/>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>Obývací stěna TERA | ŠEDÝ BETON / BÍLÁ</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>STĚNA-TERA 3/4</t>
+        </is>
+      </c>
+      <c r="C571" t="n">
+        <v>23</v>
+      </c>
+      <c r="D571" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E571" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="F571" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G571" t="inlineStr"/>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>Obývací stěna TERA | ŠEDÝ BETON / BÍLÁ</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>STĚNA-TERA 4/4</t>
+        </is>
+      </c>
+      <c r="C572" t="n">
+        <v>16</v>
+      </c>
+      <c r="D572" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="E572" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="F572" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="G572" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 24.08.2026 10:24
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G572"/>
+  <dimension ref="A1:G573"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14944,6 +14944,31 @@
       </c>
       <c r="G572" t="inlineStr"/>
     </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>Dětský povlak na polštář TROLLOVÉ</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>POVLAK</t>
+        </is>
+      </c>
+      <c r="C573" t="n">
+        <v>5</v>
+      </c>
+      <c r="D573" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E573" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F573" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G573" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 24.08.2026 10:25
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G573"/>
+  <dimension ref="A1:G574"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14969,6 +14969,31 @@
       </c>
       <c r="G573" t="inlineStr"/>
     </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>Pěnová matrace výška 9 cm KIDS COCO</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>MAT-KIDS-COCO</t>
+        </is>
+      </c>
+      <c r="C574" t="n">
+        <v>5</v>
+      </c>
+      <c r="D574" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E574" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F574" t="n">
+        <v>2</v>
+      </c>
+      <c r="G574" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 24.08.2026 10:26
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G575"/>
+  <dimension ref="A1:G576"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15019,6 +15019,31 @@
       </c>
       <c r="G575" t="inlineStr"/>
     </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>Pěnová matrace výška 10 cm EUREKA PUR</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>MAT-EUREKA</t>
+        </is>
+      </c>
+      <c r="C576" t="n">
+        <v>8</v>
+      </c>
+      <c r="D576" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E576" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F576" t="n">
+        <v>2</v>
+      </c>
+      <c r="G576" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 24.08.2026 10:28
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G577"/>
+  <dimension ref="A1:G579"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15069,6 +15069,56 @@
       </c>
       <c r="G577" t="inlineStr"/>
     </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>Dětská postel ANNITTI PINE se zábranou včetně roštu a zásuvek</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>ANNITTI-PINE 1/2</t>
+        </is>
+      </c>
+      <c r="C578" t="n">
+        <v>20</v>
+      </c>
+      <c r="D578" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E578" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F578" t="n">
+        <v>1</v>
+      </c>
+      <c r="G578" t="inlineStr"/>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>Dětská postel ANNITTI PINE se zábranou včetně roštu a zásuvek</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>ANNITTI-PINE 2/2</t>
+        </is>
+      </c>
+      <c r="C579" t="n">
+        <v>30</v>
+      </c>
+      <c r="D579" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E579" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F579" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G579" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 24.08.2026 10:29
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G579"/>
+  <dimension ref="A1:G581"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15119,6 +15119,56 @@
       </c>
       <c r="G579" t="inlineStr"/>
     </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>Dětská postel MOCHUMA se zábranou proti pádu 120x200, 140x200, 160x200 cm s roštem</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>MOCHUMA 1/2</t>
+        </is>
+      </c>
+      <c r="C580" t="n">
+        <v>21</v>
+      </c>
+      <c r="D580" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E580" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F580" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G580" t="inlineStr"/>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>Dětská postel MOCHUMA se zábranou proti pádu 120x200, 140x200, 160x200 cm s roštem</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>MOCHUMA 2/2</t>
+        </is>
+      </c>
+      <c r="C581" t="n">
+        <v>35</v>
+      </c>
+      <c r="D581" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E581" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F581" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G581" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 24.08.2026 10:31
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G581"/>
+  <dimension ref="A1:G584"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15169,6 +15169,81 @@
       </c>
       <c r="G581" t="inlineStr"/>
     </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>Patrová postel KARMA KIDBED THREE + rošty  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>KARMA-KIDBED-THREE 1/3</t>
+        </is>
+      </c>
+      <c r="C582" t="n">
+        <v>30</v>
+      </c>
+      <c r="D582" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E582" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F582" t="n">
+        <v>1</v>
+      </c>
+      <c r="G582" t="inlineStr"/>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>Patrová postel KARMA KIDBED THREE + rošty  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>KARMA-KIDBED-THREE 2/3</t>
+        </is>
+      </c>
+      <c r="C583" t="n">
+        <v>27</v>
+      </c>
+      <c r="D583" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E583" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F583" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G583" t="inlineStr"/>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>Patrová postel KARMA KIDBED THREE + rošty  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>KARMA-KIDBED-THREE 3/3</t>
+        </is>
+      </c>
+      <c r="C584" t="n">
+        <v>16</v>
+      </c>
+      <c r="D584" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E584" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F584" t="n">
+        <v>1</v>
+      </c>
+      <c r="G584" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 09.09.2026 07:33
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G584"/>
+  <dimension ref="A1:G586"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15244,6 +15244,56 @@
       </c>
       <c r="G584" t="inlineStr"/>
     </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>Rohová lavice CEZAR</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>CEZAR 1/2</t>
+        </is>
+      </c>
+      <c r="C585" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="D585" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E585" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="F585" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="G585" t="inlineStr"/>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>Rohová lavice CEZAR</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>CEZAR 2/2</t>
+        </is>
+      </c>
+      <c r="C586" t="n">
+        <v>7</v>
+      </c>
+      <c r="D586" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="E586" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="F586" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G586" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 09.09.2026 07:34
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G588"/>
+  <dimension ref="A1:G589"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15344,6 +15344,31 @@
       </c>
       <c r="G588" t="inlineStr"/>
     </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>Toaletní stolek DRESS-03</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>DRESS-03</t>
+        </is>
+      </c>
+      <c r="C589" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="D589" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E589" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="F589" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="G589" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 09.09.2026 08:13
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G589"/>
+  <dimension ref="A1:G592"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15369,6 +15369,81 @@
       </c>
       <c r="G589" t="inlineStr"/>
     </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 140x200 masiv borovice - VMK14A</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>VMK14A-140 1/3</t>
+        </is>
+      </c>
+      <c r="C590" t="n">
+        <v>18</v>
+      </c>
+      <c r="D590" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E590" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="F590" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="G590" t="inlineStr"/>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 140x200 masiv borovice - VMK14A</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>VMK14A-140 2/3</t>
+        </is>
+      </c>
+      <c r="C591" t="n">
+        <v>8</v>
+      </c>
+      <c r="D591" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="E591" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F591" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="G591" t="inlineStr"/>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 140x200 masiv borovice - VMK14A</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>VMK14A-140 3/3</t>
+        </is>
+      </c>
+      <c r="C592" t="n">
+        <v>12</v>
+      </c>
+      <c r="D592" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E592" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F592" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G592" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 21.09.2026 12:00
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H594"/>
+  <dimension ref="A1:H597"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18464,6 +18464,96 @@
         </is>
       </c>
     </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>Dětská postel s přistýlkou MAREK PINE z masivu borovice 90x200 cm včetně roštů a zábrany  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>LPW-03 1/3</t>
+        </is>
+      </c>
+      <c r="C595" t="n">
+        <v>27</v>
+      </c>
+      <c r="D595" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E595" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F595" t="n">
+        <v>1</v>
+      </c>
+      <c r="G595" t="inlineStr"/>
+      <c r="H595" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>Dětská postel s přistýlkou MAREK PINE z masivu borovice 90x200 cm včetně roštů a zábrany  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>LPW-03 2/3</t>
+        </is>
+      </c>
+      <c r="C596" t="n">
+        <v>19</v>
+      </c>
+      <c r="D596" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E596" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F596" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G596" t="inlineStr"/>
+      <c r="H596" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>Dětská postel s přistýlkou MAREK PINE z masivu borovice 90x200 cm včetně roštů a zábrany  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>LPW-03 3/3</t>
+        </is>
+      </c>
+      <c r="C597" t="n">
+        <v>24</v>
+      </c>
+      <c r="D597" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E597" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F597" t="n">
+        <v>1</v>
+      </c>
+      <c r="G597" t="inlineStr"/>
+      <c r="H597" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 21.09.2026 12:01
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H597"/>
+  <dimension ref="A1:H599"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18554,6 +18554,66 @@
         </is>
       </c>
     </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>Dětská postel z masivu se zábranou ŽOFKA PINE – včetně roštu | Borovice | Nosnost 120 kg  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>LPO-26 1/2</t>
+        </is>
+      </c>
+      <c r="C598" t="n">
+        <v>20</v>
+      </c>
+      <c r="D598" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E598" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F598" t="n">
+        <v>1</v>
+      </c>
+      <c r="G598" t="inlineStr"/>
+      <c r="H598" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>Dětská postel z masivu se zábranou ŽOFKA PINE – včetně roštu | Borovice | Nosnost 120 kg  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>LPO-26 2/2</t>
+        </is>
+      </c>
+      <c r="C599" t="n">
+        <v>28</v>
+      </c>
+      <c r="D599" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E599" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F599" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G599" t="inlineStr"/>
+      <c r="H599" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 21.09.2026 12:02
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H599"/>
+  <dimension ref="A1:H601"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18614,6 +18614,66 @@
         </is>
       </c>
     </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>Patrová postel ELPY MAX PLUS SOLID 120/140x200 vč. roštu</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>8X8-4B 1/2</t>
+        </is>
+      </c>
+      <c r="C600" t="n">
+        <v>25</v>
+      </c>
+      <c r="D600" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E600" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F600" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G600" t="inlineStr"/>
+      <c r="H600" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>Patrová postel ELPY MAX PLUS SOLID 120/140x200 vč. roštu</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>8X8-4B 2/2</t>
+        </is>
+      </c>
+      <c r="C601" t="n">
+        <v>30</v>
+      </c>
+      <c r="D601" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E601" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F601" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G601" t="inlineStr"/>
+      <c r="H601" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 21.09.2026 12:04
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H602"/>
+  <dimension ref="A1:H605"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18704,6 +18704,96 @@
         </is>
       </c>
     </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>Patrová postel ADRIANA PINE vč. roštů  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>LP-04 1/3</t>
+        </is>
+      </c>
+      <c r="C603" t="n">
+        <v>19</v>
+      </c>
+      <c r="D603" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E603" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F603" t="n">
+        <v>1</v>
+      </c>
+      <c r="G603" t="inlineStr"/>
+      <c r="H603" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>Patrová postel ADRIANA PINE vč. roštů  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>LP-04 2/3</t>
+        </is>
+      </c>
+      <c r="C604" t="n">
+        <v>27</v>
+      </c>
+      <c r="D604" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E604" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F604" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G604" t="inlineStr"/>
+      <c r="H604" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>Patrová postel ADRIANA PINE vč. roštů  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>LP-04 3/3</t>
+        </is>
+      </c>
+      <c r="C605" t="n">
+        <v>24</v>
+      </c>
+      <c r="D605" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E605" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F605" t="n">
+        <v>1</v>
+      </c>
+      <c r="G605" t="inlineStr"/>
+      <c r="H605" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 21.09.2026 12:05
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H605"/>
+  <dimension ref="A1:H607"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18794,6 +18794,66 @@
         </is>
       </c>
     </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>Dětská postel ZARA KIDBED ONE ze dřeva + rošt  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>LPO-10 1/2</t>
+        </is>
+      </c>
+      <c r="C606" t="n">
+        <v>20</v>
+      </c>
+      <c r="D606" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E606" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F606" t="n">
+        <v>1</v>
+      </c>
+      <c r="G606" t="inlineStr"/>
+      <c r="H606" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>Dětská postel ZARA KIDBED ONE ze dřeva + rošt  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>LPO-10 2/2</t>
+        </is>
+      </c>
+      <c r="C607" t="n">
+        <v>28</v>
+      </c>
+      <c r="D607" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E607" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F607" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G607" t="inlineStr"/>
+      <c r="H607" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 21.09.2026 12:08
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H607"/>
+  <dimension ref="A1:H608"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18854,6 +18854,36 @@
         </is>
       </c>
     </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>Rohový psací stůl RYDEN se zásuvkami a nástavcem 123 × 120 cm</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>INDIGO</t>
+        </is>
+      </c>
+      <c r="C608" t="n">
+        <v>50</v>
+      </c>
+      <c r="D608" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E608" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F608" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="G608" t="inlineStr"/>
+      <c r="H608" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 21.09.2026 12:12
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H609"/>
+  <dimension ref="A1:H610"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18914,6 +18914,36 @@
         </is>
       </c>
     </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>Zdravotní matrace SANJA 18 cm – ortopedická sendvičová matrace s VISCO pěnou a 7 anatomickými zónami</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>KOMODA-PREBAL-K-3+3</t>
+        </is>
+      </c>
+      <c r="C610" t="n">
+        <v>20</v>
+      </c>
+      <c r="D610" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E610" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F610" t="n">
+        <v>2</v>
+      </c>
+      <c r="G610" t="inlineStr"/>
+      <c r="H610" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 21.09.2026 12:13
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -2710,7 +2710,7 @@
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
-          <t>TOPTRANS</t>
+          <t>ALL</t>
         </is>
       </c>
     </row>
@@ -2740,7 +2740,7 @@
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
-          <t>TOPTRANS</t>
+          <t>ALL</t>
         </is>
       </c>
     </row>
@@ -2770,7 +2770,7 @@
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr">
         <is>
-          <t>TOPTRANS</t>
+          <t>ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 21.09.2026 13:25
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H610"/>
+  <dimension ref="A1:H612"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18944,6 +18944,66 @@
         </is>
       </c>
     </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 160x200 cm BOSTON z masivní borovice včetně roštu</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>BOSTON-160 1/2</t>
+        </is>
+      </c>
+      <c r="C611" t="n">
+        <v>40</v>
+      </c>
+      <c r="D611" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E611" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F611" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G611" t="inlineStr"/>
+      <c r="H611" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 160x200 cm BOSTON z masivní borovice včetně roštu</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>BOSTON-160 2/2</t>
+        </is>
+      </c>
+      <c r="C612" t="n">
+        <v>12</v>
+      </c>
+      <c r="D612" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E612" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F612" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G612" t="inlineStr"/>
+      <c r="H612" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 21.09.2026 13:26
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H612"/>
+  <dimension ref="A1:H614"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19004,6 +19004,66 @@
         </is>
       </c>
     </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>Postel BESKYD 90x200 cm z masivní borovice s roštem | Jednolůžková dřevěná postel</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>BESKYD-90 1/2</t>
+        </is>
+      </c>
+      <c r="C613" t="n">
+        <v>18</v>
+      </c>
+      <c r="D613" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E613" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F613" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G613" t="inlineStr"/>
+      <c r="H613" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>Postel BESKYD 90x200 cm z masivní borovice s roštem | Jednolůžková dřevěná postel</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>BESKYD-90 2/2</t>
+        </is>
+      </c>
+      <c r="C614" t="n">
+        <v>12</v>
+      </c>
+      <c r="D614" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E614" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F614" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G614" t="inlineStr"/>
+      <c r="H614" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 21.09.2026 13:30
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H616"/>
+  <dimension ref="A1:H618"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19124,6 +19124,66 @@
         </is>
       </c>
     </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 160x200 masiv borovice - VMK14B</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>VMK-14B-160 1/2</t>
+        </is>
+      </c>
+      <c r="C617" t="n">
+        <v>25</v>
+      </c>
+      <c r="D617" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E617" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F617" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G617" t="inlineStr"/>
+      <c r="H617" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 160x200 masiv borovice - VMK14B</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>VMK-14B-160 2/2</t>
+        </is>
+      </c>
+      <c r="C618" t="n">
+        <v>16</v>
+      </c>
+      <c r="D618" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E618" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F618" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="G618" t="inlineStr"/>
+      <c r="H618" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 21.09.2026 13:31
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H618"/>
+  <dimension ref="A1:H619"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19184,6 +19184,36 @@
         </is>
       </c>
     </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>Rošt lamelový, 80x200 cm, DOUBLE KLASIK NEW</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>DOUBLE-KLASIK-ROŠT</t>
+        </is>
+      </c>
+      <c r="C619" t="n">
+        <v>20</v>
+      </c>
+      <c r="D619" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E619" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="F619" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G619" t="inlineStr"/>
+      <c r="H619" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 22.09.2026 13:22
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H621"/>
+  <dimension ref="A1:H624"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19274,6 +19274,96 @@
         </is>
       </c>
     </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>Dětská postel s přistýlkou MONA KIDBED TWO + rošty  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>MONA-KIDBED-TWO 1/3</t>
+        </is>
+      </c>
+      <c r="C622" t="n">
+        <v>25</v>
+      </c>
+      <c r="D622" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E622" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F622" t="n">
+        <v>1</v>
+      </c>
+      <c r="G622" t="inlineStr"/>
+      <c r="H622" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>Dětská postel s přistýlkou MONA KIDBED TWO + rošty  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>MONA-KIDBED-TWO 2/3</t>
+        </is>
+      </c>
+      <c r="C623" t="n">
+        <v>20</v>
+      </c>
+      <c r="D623" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E623" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F623" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G623" t="inlineStr"/>
+      <c r="H623" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>Dětská postel s přistýlkou MONA KIDBED TWO + rošty  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>MONA-KIDBED-TWO 3/3</t>
+        </is>
+      </c>
+      <c r="C624" t="n">
+        <v>24</v>
+      </c>
+      <c r="D624" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E624" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F624" t="n">
+        <v>1</v>
+      </c>
+      <c r="G624" t="inlineStr"/>
+      <c r="H624" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 22.09.2026 13:23
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H624"/>
+  <dimension ref="A1:H626"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19364,6 +19364,66 @@
         </is>
       </c>
     </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>Dětská postel ALEXANDER PINE vč. roštu  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>ALEXANDER-PINE 1/2</t>
+        </is>
+      </c>
+      <c r="C625" t="n">
+        <v>21</v>
+      </c>
+      <c r="D625" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E625" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F625" t="n">
+        <v>1</v>
+      </c>
+      <c r="G625" t="inlineStr"/>
+      <c r="H625" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>Dětská postel ALEXANDER PINE vč. roštu  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>ALEXANDER-PINE 2/2</t>
+        </is>
+      </c>
+      <c r="C626" t="n">
+        <v>30</v>
+      </c>
+      <c r="D626" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E626" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F626" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G626" t="inlineStr"/>
+      <c r="H626" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 22.09.2026 13:24
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H626"/>
+  <dimension ref="A1:H627"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19424,6 +19424,36 @@
         </is>
       </c>
     </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>Pěnová matrace HELIOS pěna výška 20 cm</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>MAT-HELIOS</t>
+        </is>
+      </c>
+      <c r="C627" t="n">
+        <v>15</v>
+      </c>
+      <c r="D627" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E627" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F627" t="n">
+        <v>1</v>
+      </c>
+      <c r="G627" t="inlineStr"/>
+      <c r="H627" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 22.09.2026 13:25
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H627"/>
+  <dimension ref="A1:H629"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19454,6 +19454,66 @@
         </is>
       </c>
     </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 90x200 cm z masivní borovice VMK3B bezbarvý lak</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>VMK3B-90 1/2</t>
+        </is>
+      </c>
+      <c r="C628" t="n">
+        <v>12</v>
+      </c>
+      <c r="D628" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E628" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F628" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G628" t="inlineStr"/>
+      <c r="H628" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 90x200 cm z masivní borovice VMK3B bezbarvý lak</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>VMK3B-90 2/2</t>
+        </is>
+      </c>
+      <c r="C629" t="n">
+        <v>18</v>
+      </c>
+      <c r="D629" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E629" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F629" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G629" t="inlineStr"/>
+      <c r="H629" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 22.09.2026 13:27
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H629"/>
+  <dimension ref="A1:H631"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19514,6 +19514,66 @@
         </is>
       </c>
     </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 90x200 masiv borovice - VMK13B</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>VMK13B-90-1/3</t>
+        </is>
+      </c>
+      <c r="C630" t="n">
+        <v>12</v>
+      </c>
+      <c r="D630" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E630" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="F630" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G630" t="inlineStr"/>
+      <c r="H630" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 90x200 masiv borovice - VMK13B</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>VMK13B-90-2/3</t>
+        </is>
+      </c>
+      <c r="C631" t="n">
+        <v>18</v>
+      </c>
+      <c r="D631" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E631" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F631" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="G631" t="inlineStr"/>
+      <c r="H631" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 23.09.2026 11:51
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H631"/>
+  <dimension ref="A1:H632"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19574,6 +19574,36 @@
         </is>
       </c>
     </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>Dětská matrace POLO HR 10 cm – HR studená pěna H2, pratelný potah Jersey</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>MAT-POLO</t>
+        </is>
+      </c>
+      <c r="C632" t="n">
+        <v>8</v>
+      </c>
+      <c r="D632" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E632" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F632" t="n">
+        <v>2</v>
+      </c>
+      <c r="G632" t="inlineStr"/>
+      <c r="H632" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 23.09.2026 11:53
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H632"/>
+  <dimension ref="A1:H634"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19604,6 +19604,66 @@
         </is>
       </c>
     </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>Dětská postel ANNITTI PINE z masivu borovice se zábranou, roštem a zásuvkami</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>ANNITTI-PINE 1/2</t>
+        </is>
+      </c>
+      <c r="C633" t="n">
+        <v>21</v>
+      </c>
+      <c r="D633" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E633" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F633" t="n">
+        <v>1</v>
+      </c>
+      <c r="G633" t="inlineStr"/>
+      <c r="H633" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>Dětská postel ANNITTI PINE z masivu borovice se zábranou, roštem a zásuvkami</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>ANNITTI-PINE 2/2</t>
+        </is>
+      </c>
+      <c r="C634" t="n">
+        <v>30</v>
+      </c>
+      <c r="D634" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E634" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F634" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G634" t="inlineStr"/>
+      <c r="H634" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 23.09.2026 11:54
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H635"/>
+  <dimension ref="A1:H638"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19694,6 +19694,96 @@
         </is>
       </c>
     </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>Patrová postel s přistýlkou PYKE KIDBED FOUR + rošty  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>PYKE-KIDBED-FOUR 1/3</t>
+        </is>
+      </c>
+      <c r="C636" t="n">
+        <v>32</v>
+      </c>
+      <c r="D636" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E636" t="n">
+        <v>1</v>
+      </c>
+      <c r="F636" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G636" t="inlineStr"/>
+      <c r="H636" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>Patrová postel s přistýlkou PYKE KIDBED FOUR + rošty  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>PYKE-KIDBED-FOUR 2/3</t>
+        </is>
+      </c>
+      <c r="C637" t="n">
+        <v>37</v>
+      </c>
+      <c r="D637" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E637" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F637" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G637" t="inlineStr"/>
+      <c r="H637" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>Patrová postel s přistýlkou PYKE KIDBED FOUR + rošty  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>PYKE-KIDBED-FOUR 3/3</t>
+        </is>
+      </c>
+      <c r="C638" t="n">
+        <v>24</v>
+      </c>
+      <c r="D638" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E638" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F638" t="n">
+        <v>1</v>
+      </c>
+      <c r="G638" t="inlineStr"/>
+      <c r="H638" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 23.09.2026 11:55
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H638"/>
+  <dimension ref="A1:H639"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19784,6 +19784,36 @@
         </is>
       </c>
     </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>Matrace SVEA PUR 14 cm H3 – odolná pěnová matrace s pratelným potahem</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>MAT-SVEA</t>
+        </is>
+      </c>
+      <c r="C639" t="n">
+        <v>10</v>
+      </c>
+      <c r="D639" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="E639" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F639" t="n">
+        <v>2</v>
+      </c>
+      <c r="G639" t="inlineStr"/>
+      <c r="H639" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 23.09.2026 11:56
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H640"/>
+  <dimension ref="A1:H641"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19844,6 +19844,36 @@
         </is>
       </c>
     </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>Dětská matrace JUNIOR COCO 11 cm – PUR pěna T25 + kokosová vrstva, H3</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>MAT-JUNIOR-COCO</t>
+        </is>
+      </c>
+      <c r="C641" t="n">
+        <v>8</v>
+      </c>
+      <c r="D641" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="E641" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F641" t="n">
+        <v>2</v>
+      </c>
+      <c r="G641" t="inlineStr"/>
+      <c r="H641" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 23.09.2026 11:57
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H641"/>
+  <dimension ref="A1:H643"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19874,6 +19874,66 @@
         </is>
       </c>
     </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>Patrová postel TEEMO KIDBED FIVE + rošt</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>TEEMO-KIDBED-FIVE 1/2</t>
+        </is>
+      </c>
+      <c r="C642" t="n">
+        <v>22</v>
+      </c>
+      <c r="D642" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E642" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F642" t="n">
+        <v>1</v>
+      </c>
+      <c r="G642" t="inlineStr"/>
+      <c r="H642" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>Patrová postel TEEMO KIDBED FIVE + rošt</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>TEEMO-KIDBED-FIVE 2/2</t>
+        </is>
+      </c>
+      <c r="C643" t="n">
+        <v>33</v>
+      </c>
+      <c r="D643" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E643" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F643" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G643" t="inlineStr"/>
+      <c r="H643" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 23.09.2026 11:58
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H644"/>
+  <dimension ref="A1:H647"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19964,6 +19964,96 @@
         </is>
       </c>
     </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>Patrová postel BRUNO PINE vč. roštů  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>BRUNO-PINE 1/3</t>
+        </is>
+      </c>
+      <c r="C645" t="n">
+        <v>30</v>
+      </c>
+      <c r="D645" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E645" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F645" t="n">
+        <v>1</v>
+      </c>
+      <c r="G645" t="inlineStr"/>
+      <c r="H645" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>Patrová postel BRUNO PINE vč. roštů  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>BRUNO-PINE 2/3</t>
+        </is>
+      </c>
+      <c r="C646" t="n">
+        <v>27</v>
+      </c>
+      <c r="D646" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E646" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F646" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G646" t="inlineStr"/>
+      <c r="H646" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>Patrová postel BRUNO PINE vč. roštů  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>BRUNO-PINE 3/3</t>
+        </is>
+      </c>
+      <c r="C647" t="n">
+        <v>24</v>
+      </c>
+      <c r="D647" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E647" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F647" t="n">
+        <v>1</v>
+      </c>
+      <c r="G647" t="inlineStr"/>
+      <c r="H647" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 23.09.2026 11:59
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H647"/>
+  <dimension ref="A1:H648"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20054,6 +20054,36 @@
         </is>
       </c>
     </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>Pěnová matrace s kokosovou vrstvou 15 cm ADULT COCO Aloe Vera | PUR pěna T25 H3</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>MAT-ADULT-COCO</t>
+        </is>
+      </c>
+      <c r="C648" t="n">
+        <v>10</v>
+      </c>
+      <c r="D648" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E648" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F648" t="n">
+        <v>2</v>
+      </c>
+      <c r="G648" t="inlineStr"/>
+      <c r="H648" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 23.09.2026 12:00
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H650"/>
+  <dimension ref="A1:H652"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20144,6 +20144,66 @@
         </is>
       </c>
     </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>Dětská postel NIKY KIDBED ONE ze dřeva + rošt  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>NIKY-KIDBED-ONE 1/2</t>
+        </is>
+      </c>
+      <c r="C651" t="n">
+        <v>21</v>
+      </c>
+      <c r="D651" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E651" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F651" t="n">
+        <v>1</v>
+      </c>
+      <c r="G651" t="inlineStr"/>
+      <c r="H651" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>Dětská postel NIKY KIDBED ONE ze dřeva + rošt  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>NIKY-KIDBED-ONE 2/2</t>
+        </is>
+      </c>
+      <c r="C652" t="n">
+        <v>30</v>
+      </c>
+      <c r="D652" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E652" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F652" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G652" t="inlineStr"/>
+      <c r="H652" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 23.09.2026 12:01
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H652"/>
+  <dimension ref="A1:H654"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20204,6 +20204,66 @@
         </is>
       </c>
     </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 90x200 cm z masivní borovice VMK1B s roštem</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>VMK1B-90 1/2</t>
+        </is>
+      </c>
+      <c r="C653" t="n">
+        <v>18</v>
+      </c>
+      <c r="D653" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E653" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F653" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G653" t="inlineStr"/>
+      <c r="H653" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 90x200 cm z masivní borovice VMK1B s roštem</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>VMK1B-90 2/2</t>
+        </is>
+      </c>
+      <c r="C654" t="n">
+        <v>12</v>
+      </c>
+      <c r="D654" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E654" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F654" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G654" t="inlineStr"/>
+      <c r="H654" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 23.09.2026 12:02
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H654"/>
+  <dimension ref="A1:H655"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20264,6 +20264,36 @@
         </is>
       </c>
     </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>Zásuvka pod postel LK150 z masivní borovice – 97 × 85 cm</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>VMK1B-90</t>
+        </is>
+      </c>
+      <c r="C655" t="n">
+        <v>8</v>
+      </c>
+      <c r="D655" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E655" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F655" t="n">
+        <v>1</v>
+      </c>
+      <c r="G655" t="inlineStr"/>
+      <c r="H655" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 23.09.2026 12:04
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -7540,7 +7540,7 @@
       <c r="G230" t="inlineStr"/>
       <c r="H230" t="inlineStr">
         <is>
-          <t>TOPTRANS</t>
+          <t>ALL</t>
         </is>
       </c>
     </row>
@@ -7570,7 +7570,7 @@
       <c r="G231" t="inlineStr"/>
       <c r="H231" t="inlineStr">
         <is>
-          <t>TOPTRANS</t>
+          <t>ALL</t>
         </is>
       </c>
     </row>
@@ -7600,7 +7600,7 @@
       <c r="G232" t="inlineStr"/>
       <c r="H232" t="inlineStr">
         <is>
-          <t>TOPTRANS</t>
+          <t>ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 05.10.2026 13:18
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H655"/>
+  <dimension ref="A1:H657"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20294,6 +20294,66 @@
         </is>
       </c>
     </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 120x200 cm z masivní borovice VMK1B s roštem</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>VMK 1B - 120 1/2</t>
+        </is>
+      </c>
+      <c r="C656" t="n">
+        <v>18</v>
+      </c>
+      <c r="D656" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E656" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F656" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G656" t="inlineStr"/>
+      <c r="H656" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 120x200 cm z masivní borovice VMK1B s roštem</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>VMK 1B - 120 2/2</t>
+        </is>
+      </c>
+      <c r="C657" t="n">
+        <v>12</v>
+      </c>
+      <c r="D657" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E657" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F657" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="G657" t="inlineStr"/>
+      <c r="H657" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 05.10.2026 13:19
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H659"/>
+  <dimension ref="A1:H661"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20414,6 +20414,66 @@
         </is>
       </c>
     </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 120×200 cm z masivu borovice s roštem – VMK2B moření dub</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>VMK 2B - 120 1/2</t>
+        </is>
+      </c>
+      <c r="C660" t="n">
+        <v>18</v>
+      </c>
+      <c r="D660" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E660" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F660" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G660" t="inlineStr"/>
+      <c r="H660" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 120×200 cm z masivu borovice s roštem – VMK2B moření dub</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>VMK 2B - 120 2/2</t>
+        </is>
+      </c>
+      <c r="C661" t="n">
+        <v>12</v>
+      </c>
+      <c r="D661" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E661" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F661" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="G661" t="inlineStr"/>
+      <c r="H661" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 05.10.2026 13:20
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H661"/>
+  <dimension ref="A1:H663"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20474,6 +20474,66 @@
         </is>
       </c>
     </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 140x200 masiv borovice - VMK12B</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>VMK 12B - 140 1/2</t>
+        </is>
+      </c>
+      <c r="C662" t="n">
+        <v>20</v>
+      </c>
+      <c r="D662" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E662" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F662" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G662" t="inlineStr"/>
+      <c r="H662" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 140x200 masiv borovice - VMK12B</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>VMK 12B - 140 2/2</t>
+        </is>
+      </c>
+      <c r="C663" t="n">
+        <v>14</v>
+      </c>
+      <c r="D663" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E663" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F663" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="G663" t="inlineStr"/>
+      <c r="H663" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 05.10.2026 13:21
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H663"/>
+  <dimension ref="A1:H665"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20534,6 +20534,66 @@
         </is>
       </c>
     </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 120x200 cm z masivu borovice VMK3B barva bílá</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>VMK 3B - 120 1/2</t>
+        </is>
+      </c>
+      <c r="C664" t="n">
+        <v>18</v>
+      </c>
+      <c r="D664" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E664" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F664" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G664" t="inlineStr"/>
+      <c r="H664" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 120x200 cm z masivu borovice VMK3B barva bílá</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>VMK 3B - 120 2/2</t>
+        </is>
+      </c>
+      <c r="C665" t="n">
+        <v>12</v>
+      </c>
+      <c r="D665" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E665" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F665" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="G665" t="inlineStr"/>
+      <c r="H665" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 05.10.2026 13:23
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H665"/>
+  <dimension ref="A1:H667"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20594,6 +20594,66 @@
         </is>
       </c>
     </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 180x200 masiv borovice - VMK9B</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>VMK 9B - 180 1/2</t>
+        </is>
+      </c>
+      <c r="C666" t="n">
+        <v>22</v>
+      </c>
+      <c r="D666" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E666" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F666" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G666" t="inlineStr"/>
+      <c r="H666" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 180x200 masiv borovice - VMK9B</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>VMK 9B - 180 2/2</t>
+        </is>
+      </c>
+      <c r="C667" t="n">
+        <v>16</v>
+      </c>
+      <c r="D667" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E667" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F667" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="G667" t="inlineStr"/>
+      <c r="H667" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 05.10.2026 13:24
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H671"/>
+  <dimension ref="A1:H673"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20774,6 +20774,66 @@
         </is>
       </c>
     </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>Postel BESKYD 80x200 cm z masivu borovice s laťovým roštem</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>BESKYD - 80 1/2</t>
+        </is>
+      </c>
+      <c r="C672" t="n">
+        <v>14</v>
+      </c>
+      <c r="D672" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E672" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F672" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G672" t="inlineStr"/>
+      <c r="H672" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>Postel BESKYD 80x200 cm z masivu borovice s laťovým roštem</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>BESKYD - 80 2/2</t>
+        </is>
+      </c>
+      <c r="C673" t="n">
+        <v>10</v>
+      </c>
+      <c r="D673" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E673" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F673" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G673" t="inlineStr"/>
+      <c r="H673" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 05.10.2026 13:25
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H673"/>
+  <dimension ref="A1:H675"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20834,6 +20834,66 @@
         </is>
       </c>
     </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 200x200 masiv borovice - VMK8C</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>VMK 8C - 200 1/2</t>
+        </is>
+      </c>
+      <c r="C674" t="n">
+        <v>26</v>
+      </c>
+      <c r="D674" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E674" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F674" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G674" t="inlineStr"/>
+      <c r="H674" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 200x200 masiv borovice - VMK8C</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>VMK 8C - 200 2/2</t>
+        </is>
+      </c>
+      <c r="C675" t="n">
+        <v>18</v>
+      </c>
+      <c r="D675" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E675" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F675" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="G675" t="inlineStr"/>
+      <c r="H675" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 05.10.2026 13:27
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H675"/>
+  <dimension ref="A1:H677"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20894,6 +20894,66 @@
         </is>
       </c>
     </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 140x200 cm BOSTON z masivu borovice včetně roštu</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>BOSTON - 140 1/2</t>
+        </is>
+      </c>
+      <c r="C676" t="n">
+        <v>26</v>
+      </c>
+      <c r="D676" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E676" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F676" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G676" t="inlineStr"/>
+      <c r="H676" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 140x200 cm BOSTON z masivu borovice včetně roštu</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>BOSTON - 140 2/2</t>
+        </is>
+      </c>
+      <c r="C677" t="n">
+        <v>12</v>
+      </c>
+      <c r="D677" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E677" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F677" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="G677" t="inlineStr"/>
+      <c r="H677" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 05.10.2026 13:28
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H677"/>
+  <dimension ref="A1:H680"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20954,6 +20954,96 @@
         </is>
       </c>
     </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>Postel 2S, 90x200, dub sonoma, NORTY TYP 28</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>NORTY TYP 28 1/3</t>
+        </is>
+      </c>
+      <c r="C678" t="n">
+        <v>40</v>
+      </c>
+      <c r="D678" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E678" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="F678" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G678" t="inlineStr"/>
+      <c r="H678" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>Postel 2S, 90x200, dub sonoma, NORTY TYP 28</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>NORTY TYP 28 2/3</t>
+        </is>
+      </c>
+      <c r="C679" t="n">
+        <v>15</v>
+      </c>
+      <c r="D679" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="E679" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="F679" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G679" t="inlineStr"/>
+      <c r="H679" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>Postel 2S, 90x200, dub sonoma, NORTY TYP 28</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>NORTY TYP 28 3/3</t>
+        </is>
+      </c>
+      <c r="C680" t="n">
+        <v>38</v>
+      </c>
+      <c r="D680" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="E680" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="F680" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G680" t="inlineStr"/>
+      <c r="H680" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 05.10.2026 13:30
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H680"/>
+  <dimension ref="A1:H681"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21044,6 +21044,36 @@
         </is>
       </c>
     </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>Zásuvka / šuplík pod postel LK152, 197 × 65 cm, masivní borovice</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>ZÁSUVKA LK152</t>
+        </is>
+      </c>
+      <c r="C681" t="n">
+        <v>20</v>
+      </c>
+      <c r="D681" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E681" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F681" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="G681" t="inlineStr"/>
+      <c r="H681" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 05.10.2026 13:32
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H681"/>
+  <dimension ref="A1:H684"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21074,6 +21074,96 @@
         </is>
       </c>
     </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>Dětská postel s přistýlkou MONIKA PINE vč. roštů | 90 x 200 cm, barva modrá  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>MONIKA PINE 1/3</t>
+        </is>
+      </c>
+      <c r="C682" t="n">
+        <v>21</v>
+      </c>
+      <c r="D682" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E682" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F682" t="n">
+        <v>1</v>
+      </c>
+      <c r="G682" t="inlineStr"/>
+      <c r="H682" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>Dětská postel s přistýlkou MONIKA PINE vč. roštů | 90 x 200 cm, barva modrá  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>MONIKA PINE 2/3</t>
+        </is>
+      </c>
+      <c r="C683" t="n">
+        <v>20</v>
+      </c>
+      <c r="D683" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E683" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F683" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G683" t="inlineStr"/>
+      <c r="H683" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>Dětská postel s přistýlkou MONIKA PINE vč. roštů | 90 x 200 cm, barva modrá  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>MONIKA PINE 3/3</t>
+        </is>
+      </c>
+      <c r="C684" t="n">
+        <v>24</v>
+      </c>
+      <c r="D684" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E684" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F684" t="n">
+        <v>1</v>
+      </c>
+      <c r="G684" t="inlineStr"/>
+      <c r="H684" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 05.10.2026 13:33
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H684"/>
+  <dimension ref="A1:H687"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21164,6 +21164,96 @@
         </is>
       </c>
     </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>Dětská postel s přistýlkou MAREK PINE z masivu borovice 90x200 cm včetně roštů  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>MAREK PINE 1/3</t>
+        </is>
+      </c>
+      <c r="C685" t="n">
+        <v>25</v>
+      </c>
+      <c r="D685" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E685" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F685" t="n">
+        <v>1</v>
+      </c>
+      <c r="G685" t="inlineStr"/>
+      <c r="H685" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>Dětská postel s přistýlkou MAREK PINE z masivu borovice 90x200 cm včetně roštů  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>MAREK PINE 2/3</t>
+        </is>
+      </c>
+      <c r="C686" t="n">
+        <v>20</v>
+      </c>
+      <c r="D686" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E686" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F686" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G686" t="inlineStr"/>
+      <c r="H686" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>Dětská postel s přistýlkou MAREK PINE z masivu borovice 90x200 cm včetně roštů  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>MAREK PINE 3/3</t>
+        </is>
+      </c>
+      <c r="C687" t="n">
+        <v>24</v>
+      </c>
+      <c r="D687" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E687" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F687" t="n">
+        <v>1</v>
+      </c>
+      <c r="G687" t="inlineStr"/>
+      <c r="H687" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 05.10.2026 13:34
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -21262,7 +21262,7 @@
       </c>
       <c r="B688" t="inlineStr">
         <is>
-          <t>MAREK PINE 1/3</t>
+          <t>JUNIOR PLUS 1/3</t>
         </is>
       </c>
       <c r="C688" t="n">
@@ -21292,7 +21292,7 @@
       </c>
       <c r="B689" t="inlineStr">
         <is>
-          <t>MAREK PINE 2/3</t>
+          <t>JUNIOR PLUS 2/3</t>
         </is>
       </c>
       <c r="C689" t="n">
@@ -21322,7 +21322,7 @@
       </c>
       <c r="B690" t="inlineStr">
         <is>
-          <t>MAREK PINE 3/3</t>
+          <t>JUNIOR PLUS 3/3</t>
         </is>
       </c>
       <c r="C690" t="n">

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 05.10.2026 13:35
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H690"/>
+  <dimension ref="A1:H691"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21344,6 +21344,36 @@
         </is>
       </c>
     </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>Zásuvka pod postel LK151, masivní borovice, 150 × 85 cm</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>ZÁSUVKA LK151</t>
+        </is>
+      </c>
+      <c r="C691" t="n">
+        <v>18</v>
+      </c>
+      <c r="D691" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E691" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F691" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="G691" t="inlineStr"/>
+      <c r="H691" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 05.10.2026 13:36
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H691"/>
+  <dimension ref="A1:H693"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21374,6 +21374,66 @@
         </is>
       </c>
     </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>Patrová postel KL-135</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>POSTEL KL-135 1/2</t>
+        </is>
+      </c>
+      <c r="C692" t="n">
+        <v>35</v>
+      </c>
+      <c r="D692" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E692" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F692" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G692" t="inlineStr"/>
+      <c r="H692" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>Patrová postel KL-135</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>POSTEL KL-135 2/2</t>
+        </is>
+      </c>
+      <c r="C693" t="n">
+        <v>28</v>
+      </c>
+      <c r="D693" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E693" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F693" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G693" t="inlineStr"/>
+      <c r="H693" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 05.10.2026 13:37
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H693"/>
+  <dimension ref="A1:H695"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21434,6 +21434,66 @@
         </is>
       </c>
     </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>Postel LENA 90x200 | MASIV BOROVICE</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>LENA-90X200 1/2</t>
+        </is>
+      </c>
+      <c r="C694" t="n">
+        <v>15</v>
+      </c>
+      <c r="D694" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E694" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F694" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="G694" t="inlineStr"/>
+      <c r="H694" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>Postel LENA 90x200 | MASIV BOROVICE</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>LENA-90X200 2/3</t>
+        </is>
+      </c>
+      <c r="C695" t="n">
+        <v>10</v>
+      </c>
+      <c r="D695" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E695" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F695" t="n">
+        <v>2</v>
+      </c>
+      <c r="G695" t="inlineStr"/>
+      <c r="H695" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 06.10.2026 11:24
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H695"/>
+  <dimension ref="A1:H697"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21494,6 +21494,66 @@
         </is>
       </c>
     </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>Rohová jídelní lavice JENARAE</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>ROHOVÁ LAVICE JENARAE 1/2</t>
+        </is>
+      </c>
+      <c r="C696" t="n">
+        <v>32</v>
+      </c>
+      <c r="D696" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E696" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F696" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="G696" t="inlineStr"/>
+      <c r="H696" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>Rohová jídelní lavice JENARAE</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>ROHOVÁ LAVICE JENARAE 2/2</t>
+        </is>
+      </c>
+      <c r="C697" t="n">
+        <v>7</v>
+      </c>
+      <c r="D697" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="E697" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="F697" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G697" t="inlineStr"/>
+      <c r="H697" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 06.10.2026 11:25
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H697"/>
+  <dimension ref="A1:H701"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21554,6 +21554,126 @@
         </is>
       </c>
     </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>Jídelní rohový set JOKULL dub kraft / koženka bílá</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>SET JOKULL 1/4</t>
+        </is>
+      </c>
+      <c r="C698" t="n">
+        <v>23</v>
+      </c>
+      <c r="D698" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="E698" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="F698" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="G698" t="inlineStr"/>
+      <c r="H698" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>Jídelní rohový set JOKULL dub kraft / koženka bílá</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>SET JOKULL 2/4</t>
+        </is>
+      </c>
+      <c r="C699" t="n">
+        <v>6</v>
+      </c>
+      <c r="D699" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="E699" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="F699" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="G699" t="inlineStr"/>
+      <c r="H699" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>Jídelní rohový set JOKULL dub kraft / koženka bílá</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>SET JOKULL 3/4</t>
+        </is>
+      </c>
+      <c r="C700" t="n">
+        <v>12</v>
+      </c>
+      <c r="D700" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E700" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="F700" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="G700" t="inlineStr"/>
+      <c r="H700" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>Jídelní rohový set JOKULL dub kraft / koženka bílá</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>SET JOKULL 4/4</t>
+        </is>
+      </c>
+      <c r="C701" t="n">
+        <v>7</v>
+      </c>
+      <c r="D701" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="E701" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="F701" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="G701" t="inlineStr"/>
+      <c r="H701" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 06.10.2026 11:26
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H701"/>
+  <dimension ref="A1:H702"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21674,6 +21674,36 @@
         </is>
       </c>
     </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>Komoda LATHAM SX-03 nízká s posuvnými dvířky a policovým prostorem</t>
+        </is>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>KOMODA LATHAM SX-03</t>
+        </is>
+      </c>
+      <c r="C702" t="n">
+        <v>24</v>
+      </c>
+      <c r="D702" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E702" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="F702" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="G702" t="inlineStr"/>
+      <c r="H702" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 06.10.2026 11:27
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H702"/>
+  <dimension ref="A1:H704"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21704,6 +21704,66 @@
         </is>
       </c>
     </row>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 90x200 borovice VMK5C bezbarvý lak</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>VMK 5C - 90 1/2</t>
+        </is>
+      </c>
+      <c r="C703" t="n">
+        <v>18</v>
+      </c>
+      <c r="D703" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E703" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F703" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G703" t="inlineStr"/>
+      <c r="H703" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 90x200 borovice VMK5C bezbarvý lak</t>
+        </is>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>VMK 5C - 90 2/2</t>
+        </is>
+      </c>
+      <c r="C704" t="n">
+        <v>10</v>
+      </c>
+      <c r="D704" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E704" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F704" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G704" t="inlineStr"/>
+      <c r="H704" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 06.10.2026 11:28
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H704"/>
+  <dimension ref="A1:H706"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21764,6 +21764,66 @@
         </is>
       </c>
     </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 120×200 cm z masivu borovice s roštem – VMK2B bezbarvý lak</t>
+        </is>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>VMK 2B - 120 1/2</t>
+        </is>
+      </c>
+      <c r="C705" t="n">
+        <v>20</v>
+      </c>
+      <c r="D705" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E705" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F705" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G705" t="inlineStr"/>
+      <c r="H705" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 120×200 cm z masivu borovice s roštem – VMK2B bezbarvý lak</t>
+        </is>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>VMK 2B - 120 2/2</t>
+        </is>
+      </c>
+      <c r="C706" t="n">
+        <v>12</v>
+      </c>
+      <c r="D706" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E706" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F706" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="G706" t="inlineStr"/>
+      <c r="H706" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 08.10.2026 09:42
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H706"/>
+  <dimension ref="A1:H707"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21824,6 +21824,36 @@
         </is>
       </c>
     </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>Konferenční stolek rozkládací BASILE</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>stolek BASILE</t>
+        </is>
+      </c>
+      <c r="C707" t="n">
+        <v>16</v>
+      </c>
+      <c r="D707" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="E707" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="F707" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="G707" t="inlineStr"/>
+      <c r="H707" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 08.10.2026 09:43
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H708"/>
+  <dimension ref="A1:H709"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21884,6 +21884,36 @@
         </is>
       </c>
     </row>
+    <row r="709">
+      <c r="A709" t="inlineStr">
+        <is>
+          <t>Závěsná police MX-13</t>
+        </is>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>regál LATHAM-06</t>
+        </is>
+      </c>
+      <c r="C709" t="n">
+        <v>8</v>
+      </c>
+      <c r="D709" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="E709" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F709" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G709" t="inlineStr"/>
+      <c r="H709" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 08.10.2026 09:44
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H709"/>
+  <dimension ref="A1:H710"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21914,6 +21914,36 @@
         </is>
       </c>
     </row>
+    <row r="710">
+      <c r="A710" t="inlineStr">
+        <is>
+          <t>Sedací botník DEYLIS se sedákem, policemi na boty a úložným prostorem do předsíně</t>
+        </is>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>botník DEYLIS</t>
+        </is>
+      </c>
+      <c r="C710" t="n">
+        <v>26</v>
+      </c>
+      <c r="D710" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="E710" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="F710" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="G710" t="inlineStr"/>
+      <c r="H710" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 08.10.2026 09:45
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H710"/>
+  <dimension ref="A1:H712"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21944,6 +21944,66 @@
         </is>
       </c>
     </row>
+    <row r="711">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>Komoda-8 BLAISE NEW</t>
+        </is>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>komoda-8 BLAISE NEW 1/2</t>
+        </is>
+      </c>
+      <c r="C711" t="n">
+        <v>27</v>
+      </c>
+      <c r="D711" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="E711" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F711" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="G711" t="inlineStr"/>
+      <c r="H711" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>Komoda-8 BLAISE NEW</t>
+        </is>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>komoda-8 BLAISE NEW 2/2</t>
+        </is>
+      </c>
+      <c r="C712" t="n">
+        <v>29</v>
+      </c>
+      <c r="D712" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E712" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F712" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="G712" t="inlineStr"/>
+      <c r="H712" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 08.10.2026 09:46
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H712"/>
+  <dimension ref="A1:H713"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22004,6 +22004,36 @@
         </is>
       </c>
     </row>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>Televizní stolek DELVIN</t>
+        </is>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>stolek DELVIN</t>
+        </is>
+      </c>
+      <c r="C713" t="n">
+        <v>32</v>
+      </c>
+      <c r="D713" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="E713" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="F713" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="G713" t="inlineStr"/>
+      <c r="H713" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 08.10.2026 09:47
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H713"/>
+  <dimension ref="A1:H714"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22034,6 +22034,36 @@
         </is>
       </c>
     </row>
+    <row r="714">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>Jídelní stůl SN-04 80 × 60 cm – kompaktní stůl do kuchyně a jídelny</t>
+        </is>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>stůl SN-04</t>
+        </is>
+      </c>
+      <c r="C714" t="n">
+        <v>12</v>
+      </c>
+      <c r="D714" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E714" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="F714" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="G714" t="inlineStr"/>
+      <c r="H714" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 08.10.2026 09:48
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H715"/>
+  <dimension ref="A1:H716"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22094,6 +22094,36 @@
         </is>
       </c>
     </row>
+    <row r="716">
+      <c r="A716" t="inlineStr">
+        <is>
+          <t>Rohová jídelní lavice HAROLD s úložným prostorem 150 × 110 cm – univerzální pravá/levá varianta</t>
+        </is>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>lavice HAROLD</t>
+        </is>
+      </c>
+      <c r="C716" t="n">
+        <v>42</v>
+      </c>
+      <c r="D716" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="E716" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="F716" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="G716" t="inlineStr"/>
+      <c r="H716" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 08.10.2026 09:49
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H716"/>
+  <dimension ref="A1:H720"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22124,6 +22124,126 @@
         </is>
       </c>
     </row>
+    <row r="717">
+      <c r="A717" t="inlineStr">
+        <is>
+          <t>Jídelní rohový set JENARAE dub tacho - koženka hnědá</t>
+        </is>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>rohový set JANARAE 1/4</t>
+        </is>
+      </c>
+      <c r="C717" t="n">
+        <v>32</v>
+      </c>
+      <c r="D717" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E717" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F717" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="G717" t="inlineStr"/>
+      <c r="H717" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="inlineStr">
+        <is>
+          <t>Jídelní rohový set JENARAE dub tacho - koženka hnědá</t>
+        </is>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>rohový set JANARAE 2/4</t>
+        </is>
+      </c>
+      <c r="C718" t="n">
+        <v>7</v>
+      </c>
+      <c r="D718" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="E718" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="F718" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G718" t="inlineStr"/>
+      <c r="H718" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="inlineStr">
+        <is>
+          <t>Jídelní rohový set JENARAE dub tacho - koženka hnědá</t>
+        </is>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>rohový set JANARAE 3/4</t>
+        </is>
+      </c>
+      <c r="C719" t="n">
+        <v>21</v>
+      </c>
+      <c r="D719" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="E719" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="F719" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="G719" t="inlineStr"/>
+      <c r="H719" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>Jídelní rohový set JENARAE dub tacho - koženka hnědá</t>
+        </is>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>rohový set JANARAE 4/4</t>
+        </is>
+      </c>
+      <c r="C720" t="n">
+        <v>8</v>
+      </c>
+      <c r="D720" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E720" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="F720" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="G720" t="inlineStr"/>
+      <c r="H720" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 08.10.2026 09:50
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H720"/>
+  <dimension ref="A1:H721"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22244,6 +22244,36 @@
         </is>
       </c>
     </row>
+    <row r="721">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>Jídelní židle ARIANNA šedá – čalouněná jídelní židle s ocelovou konstrukcí</t>
+        </is>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>židle ARIANNA</t>
+        </is>
+      </c>
+      <c r="C721" t="n">
+        <v>8</v>
+      </c>
+      <c r="D721" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E721" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F721" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G721" t="inlineStr"/>
+      <c r="H721" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 08.10.2026 09:53
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H721"/>
+  <dimension ref="A1:H722"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22274,6 +22274,36 @@
         </is>
       </c>
     </row>
+    <row r="722">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>Noční stolek BOGAN NEW 1S bílý</t>
+        </is>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>NČ BOGAN NEW</t>
+        </is>
+      </c>
+      <c r="C722" t="n">
+        <v>11</v>
+      </c>
+      <c r="D722" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E722" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="F722" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="G722" t="inlineStr"/>
+      <c r="H722" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 12.10.2026 12:34
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H722"/>
+  <dimension ref="A1:H724"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22304,6 +22304,66 @@
         </is>
       </c>
     </row>
+    <row r="723">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>Televizní stolek DOMINIC</t>
+        </is>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>stolek DOMINIC 1/2</t>
+        </is>
+      </c>
+      <c r="C723" t="n">
+        <v>25</v>
+      </c>
+      <c r="D723" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E723" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="F723" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="G723" t="inlineStr"/>
+      <c r="H723" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>Televizní stolek DOMINIC</t>
+        </is>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>stolek DOMINIC 2/2</t>
+        </is>
+      </c>
+      <c r="C724" t="n">
+        <v>10</v>
+      </c>
+      <c r="D724" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E724" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="F724" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="G724" t="inlineStr"/>
+      <c r="H724" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 12.10.2026 12:35
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H724"/>
+  <dimension ref="A1:H725"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22364,6 +22364,36 @@
         </is>
       </c>
     </row>
+    <row r="725">
+      <c r="A725" t="inlineStr">
+        <is>
+          <t>Výklopný botník MARCOS se zásuvkou a regálem – úzký dvouřadý botník do předsíně 80 × 117 × 25 cm</t>
+        </is>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>botník MARCOS</t>
+        </is>
+      </c>
+      <c r="C725" t="n">
+        <v>31</v>
+      </c>
+      <c r="D725" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="E725" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="F725" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="G725" t="inlineStr"/>
+      <c r="H725" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 12.10.2026 12:36
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H725"/>
+  <dimension ref="A1:H726"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22394,6 +22394,36 @@
         </is>
       </c>
     </row>
+    <row r="726">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>Botník KENDALL 80 cm – policový regál na boty do předsíně, 80 × 68 × 27 cm</t>
+        </is>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>botník KENDALL</t>
+        </is>
+      </c>
+      <c r="C726" t="n">
+        <v>16</v>
+      </c>
+      <c r="D726" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E726" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="F726" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G726" t="inlineStr"/>
+      <c r="H726" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 12.10.2026 12:39
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H728"/>
+  <dimension ref="A1:H729"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22484,6 +22484,36 @@
         </is>
       </c>
     </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>Rozkládací pohovka ALISIA šedohnědá Taupe / gold chrom zlatý</t>
+        </is>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>pohovka ALISIA</t>
+        </is>
+      </c>
+      <c r="C729" t="n">
+        <v>34</v>
+      </c>
+      <c r="D729" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="E729" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="F729" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="G729" t="inlineStr"/>
+      <c r="H729" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 12.10.2026 12:40
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H729"/>
+  <dimension ref="A1:H731"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22514,6 +22514,66 @@
         </is>
       </c>
     </row>
+    <row r="730">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>Policový botník MARC dub sonoma – vysoký úzký regál na boty s otevřenými policemi 180 cm</t>
+        </is>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>botník MARC 1/2</t>
+        </is>
+      </c>
+      <c r="C730" t="n">
+        <v>15</v>
+      </c>
+      <c r="D730" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E730" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="F730" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="G730" t="inlineStr"/>
+      <c r="H730" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>Policový botník MARC dub sonoma – vysoký úzký regál na boty s otevřenými policemi 180 cm</t>
+        </is>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>botník MARC 2/2</t>
+        </is>
+      </c>
+      <c r="C731" t="n">
+        <v>24</v>
+      </c>
+      <c r="D731" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E731" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F731" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="G731" t="inlineStr"/>
+      <c r="H731" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aktualizace katalogu produktů - 12.10.2026 12:42
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H732"/>
+  <dimension ref="A1:H736"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22604,6 +22604,126 @@
         </is>
       </c>
     </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>Patrová postel RUDI PINE vč. roštů  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>RUDI PINE 1/4</t>
+        </is>
+      </c>
+      <c r="C733" t="n">
+        <v>27</v>
+      </c>
+      <c r="D733" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E733" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F733" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G733" t="inlineStr"/>
+      <c r="H733" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>Patrová postel RUDI PINE vč. roštů  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>RUDI PINE 2/4</t>
+        </is>
+      </c>
+      <c r="C734" t="n">
+        <v>19</v>
+      </c>
+      <c r="D734" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E734" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F734" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G734" t="inlineStr"/>
+      <c r="H734" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>Patrová postel RUDI PINE vč. roštů  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>RUDI PINE 3/4</t>
+        </is>
+      </c>
+      <c r="C735" t="n">
+        <v>31</v>
+      </c>
+      <c r="D735" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E735" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="F735" t="n">
+        <v>1</v>
+      </c>
+      <c r="G735" t="inlineStr"/>
+      <c r="H735" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>Patrová postel RUDI PINE vč. roštů  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>RUDI PINE 4/4</t>
+        </is>
+      </c>
+      <c r="C736" t="n">
+        <v>5</v>
+      </c>
+      <c r="D736" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E736" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F736" t="n">
+        <v>1</v>
+      </c>
+      <c r="G736" t="inlineStr"/>
+      <c r="H736" t="inlineStr">
+        <is>
+          <t>NOVAPOST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>